<commit_message>
feat: Siparis Ayirma & Akilli Hat Dagitim Motoru entegrasyonu (2 veya daha fazla hatta eszamanli bolusturme, en ideal 2 hat tavsiye motoru)
</commit_message>
<xml_diff>
--- a/static/Ergunbas_Ekstruzyon_ve_Kalite_Kontrol_Vardiya_Kapasite_Matrisi.xlsx
+++ b/static/Ergunbas_Ekstruzyon_ve_Kalite_Kontrol_Vardiya_Kapasite_Matrisi.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Ürün Detaylı Kapasite Matrisi" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ürün Detaylı Kapasite Matrisi'!$A$4:$Q$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ürün Detaylı Kapasite Matrisi'!$A$4:$Q$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -182,7 +182,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -328,15 +328,6 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="169" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="170" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1389,7 +1380,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q42"/>
+  <dimension ref="A1:Q32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1582,14 +1573,14 @@
         <v>244</v>
       </c>
       <c r="N5" s="34" t="n">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="O5" s="35" t="n">
-        <v>1071.4</v>
+        <v>1073.6</v>
       </c>
       <c r="P5" s="36" t="inlineStr">
         <is>
-          <t>97 Kapı/Gün</t>
+          <t>98 Kapı/Gün</t>
         </is>
       </c>
       <c r="Q5" s="37" t="inlineStr">
@@ -1655,10 +1646,10 @@
         <v>262</v>
       </c>
       <c r="N6" s="44" t="n">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="O6" s="45" t="n">
-        <v>1087.8</v>
+        <v>1089.9</v>
       </c>
       <c r="P6" s="46" t="inlineStr">
         <is>
@@ -2016,10 +2007,10 @@
         <v>398</v>
       </c>
       <c r="N11" s="34" t="n">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="O11" s="35" t="n">
-        <v>1195.5</v>
+        <v>1194</v>
       </c>
       <c r="P11" s="36" t="inlineStr">
         <is>
@@ -2089,10 +2080,10 @@
         <v>1024</v>
       </c>
       <c r="N12" s="44" t="n">
-        <v>2047</v>
+        <v>2048</v>
       </c>
       <c r="O12" s="45" t="n">
-        <v>982.6</v>
+        <v>983</v>
       </c>
       <c r="P12" s="6" t="inlineStr">
         <is>
@@ -2300,10 +2291,10 @@
         <v>338</v>
       </c>
       <c r="N15" s="34" t="n">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="O15" s="35" t="n">
-        <v>2295</v>
+        <v>2291.6</v>
       </c>
       <c r="P15" s="36" t="inlineStr">
         <is>
@@ -2369,10 +2360,10 @@
         <v>320</v>
       </c>
       <c r="N16" s="44" t="n">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="O16" s="45" t="n">
-        <v>2173</v>
+        <v>2169.6</v>
       </c>
       <c r="P16" s="46" t="inlineStr">
         <is>
@@ -2872,10 +2863,10 @@
         <v>98</v>
       </c>
       <c r="N23" s="34" t="n">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="O23" s="35" t="n">
-        <v>2035</v>
+        <v>2024.7</v>
       </c>
       <c r="P23" s="14" t="inlineStr">
         <is>
@@ -2945,10 +2936,10 @@
         <v>124</v>
       </c>
       <c r="N24" s="44" t="n">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="O24" s="45" t="n">
-        <v>2598.4</v>
+        <v>2609</v>
       </c>
       <c r="P24" s="6" t="inlineStr">
         <is>
@@ -3087,10 +3078,10 @@
         <v>206</v>
       </c>
       <c r="N26" s="44" t="n">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="O26" s="45" t="n">
-        <v>1652</v>
+        <v>1648</v>
       </c>
       <c r="P26" s="46" t="inlineStr">
         <is>
@@ -3160,10 +3151,10 @@
         <v>176</v>
       </c>
       <c r="N27" s="34" t="n">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="O27" s="35" t="n">
-        <v>1747.4</v>
+        <v>1742.4</v>
       </c>
       <c r="P27" s="36" t="inlineStr">
         <is>
@@ -3229,10 +3220,10 @@
         <v>584</v>
       </c>
       <c r="N28" s="44" t="n">
-        <v>1169</v>
+        <v>1168</v>
       </c>
       <c r="O28" s="45" t="n">
-        <v>1812</v>
+        <v>1810.4</v>
       </c>
       <c r="P28" s="46" t="inlineStr">
         <is>
@@ -3343,7 +3334,7 @@
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>DIŞBUDAK Levha</t>
+          <t>WPC Kapı Levhası (Genel Ortalama)</t>
         </is>
       </c>
       <c r="H30" s="9" t="inlineStr">
@@ -3362,40 +3353,40 @@
         </is>
       </c>
       <c r="K30" s="41" t="n">
-        <v>4.77</v>
+        <v>4.58</v>
       </c>
       <c r="L30" s="48" t="n">
-        <v>42.7</v>
+        <v>41.7</v>
       </c>
       <c r="M30" s="49" t="n">
-        <v>512</v>
+        <v>500</v>
       </c>
       <c r="N30" s="50" t="n">
-        <v>1025</v>
+        <v>1000</v>
       </c>
       <c r="O30" s="45" t="n">
-        <v>4889.2</v>
+        <v>4580</v>
       </c>
       <c r="P30" s="46" t="inlineStr">
         <is>
-          <t>512 Kapı/Gün</t>
+          <t>500 Kapı/Gün</t>
         </is>
       </c>
       <c r="Q30" s="38" t="inlineStr">
         <is>
-          <t>En Yüksek Hacim</t>
+          <t>Tüm Renkler Genel Ortalaması</t>
         </is>
       </c>
     </row>
     <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="37" t="inlineStr">
-        <is>
-          <t>↳ Hat 201 (Levha)</t>
+      <c r="A31" s="12" t="inlineStr">
+        <is>
+          <t>KALİTE KONTROL</t>
         </is>
       </c>
       <c r="B31" s="13" t="inlineStr">
         <is>
-          <t>20:30 / 08:30</t>
+          <t>08:30 / 20:30 (2V)</t>
         </is>
       </c>
       <c r="C31" s="28" t="n">
@@ -3404,823 +3395,93 @@
       <c r="D31" s="29" t="n">
         <v>720</v>
       </c>
-      <c r="E31" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F31" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="E31" s="30" t="n">
+        <v>3</v>
+      </c>
+      <c r="F31" s="30" t="n">
+        <v>3</v>
       </c>
       <c r="G31" s="12" t="inlineStr">
         <is>
-          <t>TEAK Levha</t>
+          <t>TÜM PROFİL &amp; LEVHALAR</t>
         </is>
       </c>
       <c r="H31" s="17" t="inlineStr">
         <is>
-          <t>WPC Levha Plaka</t>
+          <t>Kalite Güvence</t>
         </is>
       </c>
       <c r="I31" s="10" t="inlineStr">
         <is>
-          <t>2.07 m</t>
+          <t>Tüm Boylar</t>
         </is>
       </c>
       <c r="J31" s="17" t="inlineStr">
         <is>
-          <t>En: 94 cm (2 mm)</t>
-        </is>
-      </c>
-      <c r="K31" s="31" t="n">
-        <v>4.25</v>
+          <t>Tüm Kesitler</t>
+        </is>
+      </c>
+      <c r="K31" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="L31" s="51" t="n">
-        <v>38.6</v>
+        <v>175</v>
       </c>
       <c r="M31" s="52" t="n">
-        <v>463</v>
+        <v>2100</v>
       </c>
       <c r="N31" s="53" t="n">
-        <v>926</v>
-      </c>
-      <c r="O31" s="35" t="n">
-        <v>3935.5</v>
-      </c>
-      <c r="P31" s="36" t="inlineStr">
-        <is>
-          <t>463 Kapı/Gün</t>
+        <v>4200</v>
+      </c>
+      <c r="O31" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P31" s="14" t="inlineStr">
+        <is>
+          <t>4.200 Adet/Gün</t>
         </is>
       </c>
       <c r="Q31" s="37" t="inlineStr">
         <is>
-          <t>Seri Üretim</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="38" t="inlineStr">
-        <is>
-          <t>↳ Hat 201 (Levha)</t>
-        </is>
-      </c>
-      <c r="B32" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C32" s="39" t="n">
-        <v>720</v>
-      </c>
-      <c r="D32" s="40" t="n">
-        <v>720</v>
-      </c>
-      <c r="E32" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F32" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G32" s="4" t="inlineStr">
-        <is>
-          <t>MIX TEAK Levha</t>
-        </is>
-      </c>
-      <c r="H32" s="9" t="inlineStr">
-        <is>
-          <t>WPC Levha Plaka</t>
-        </is>
-      </c>
-      <c r="I32" s="10" t="inlineStr">
-        <is>
-          <t>2.07 m</t>
-        </is>
-      </c>
-      <c r="J32" s="9" t="inlineStr">
-        <is>
-          <t>En: 94 cm (2 mm)</t>
-        </is>
-      </c>
-      <c r="K32" s="41" t="n">
-        <v>4.25</v>
-      </c>
-      <c r="L32" s="48" t="n">
-        <v>40.1</v>
-      </c>
-      <c r="M32" s="49" t="n">
-        <v>481</v>
-      </c>
-      <c r="N32" s="50" t="n">
-        <v>962</v>
-      </c>
-      <c r="O32" s="45" t="n">
-        <v>4088.5</v>
-      </c>
-      <c r="P32" s="46" t="inlineStr">
-        <is>
-          <t>481 Kapı/Gün</t>
-        </is>
-      </c>
-      <c r="Q32" s="38" t="inlineStr">
-        <is>
-          <t>Seri Üretim</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="20" customHeight="1">
-      <c r="A33" s="37" t="inlineStr">
-        <is>
-          <t>↳ Hat 201 (Levha)</t>
-        </is>
-      </c>
-      <c r="B33" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C33" s="28" t="n">
-        <v>720</v>
-      </c>
-      <c r="D33" s="29" t="n">
-        <v>720</v>
-      </c>
-      <c r="E33" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F33" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G33" s="12" t="inlineStr">
-        <is>
-          <t>BEYAZ TEAK Levha</t>
-        </is>
-      </c>
-      <c r="H33" s="17" t="inlineStr">
-        <is>
-          <t>WPC Levha Plaka</t>
-        </is>
-      </c>
-      <c r="I33" s="10" t="inlineStr">
-        <is>
-          <t>2.07 m</t>
-        </is>
-      </c>
-      <c r="J33" s="17" t="inlineStr">
-        <is>
-          <t>En: 94 cm (2 mm)</t>
-        </is>
-      </c>
-      <c r="K33" s="31" t="n">
-        <v>4.41</v>
-      </c>
-      <c r="L33" s="51" t="n">
-        <v>40.6</v>
-      </c>
-      <c r="M33" s="52" t="n">
-        <v>487</v>
-      </c>
-      <c r="N33" s="53" t="n">
-        <v>974</v>
-      </c>
-      <c r="O33" s="35" t="n">
-        <v>4295.3</v>
-      </c>
-      <c r="P33" s="36" t="inlineStr">
-        <is>
-          <t>487 Kapı/Gün</t>
-        </is>
-      </c>
-      <c r="Q33" s="37" t="inlineStr">
-        <is>
-          <t>Seri Üretim</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="38" t="inlineStr">
-        <is>
-          <t>↳ Hat 201 (Levha)</t>
-        </is>
-      </c>
-      <c r="B34" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C34" s="39" t="n">
-        <v>720</v>
-      </c>
-      <c r="D34" s="40" t="n">
-        <v>720</v>
-      </c>
-      <c r="E34" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F34" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G34" s="4" t="inlineStr">
-        <is>
-          <t>MIX BEYAZ TEAK Levha</t>
-        </is>
-      </c>
-      <c r="H34" s="9" t="inlineStr">
-        <is>
-          <t>WPC Levha Plaka</t>
-        </is>
-      </c>
-      <c r="I34" s="10" t="inlineStr">
-        <is>
-          <t>2.07 m</t>
-        </is>
-      </c>
-      <c r="J34" s="9" t="inlineStr">
-        <is>
-          <t>En: 94 cm (2 mm)</t>
-        </is>
-      </c>
-      <c r="K34" s="41" t="n">
-        <v>4.25</v>
-      </c>
-      <c r="L34" s="48" t="n">
-        <v>44.1</v>
-      </c>
-      <c r="M34" s="49" t="n">
-        <v>529</v>
-      </c>
-      <c r="N34" s="50" t="n">
-        <v>1058</v>
-      </c>
-      <c r="O34" s="45" t="n">
-        <v>4496.5</v>
-      </c>
-      <c r="P34" s="46" t="inlineStr">
-        <is>
-          <t>529 Kapı/Gün</t>
-        </is>
-      </c>
-      <c r="Q34" s="38" t="inlineStr">
-        <is>
-          <t>Yüksek Hızlı</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="37" t="inlineStr">
-        <is>
-          <t>↳ Hat 201 (Levha)</t>
-        </is>
-      </c>
-      <c r="B35" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C35" s="28" t="n">
-        <v>720</v>
-      </c>
-      <c r="D35" s="29" t="n">
-        <v>720</v>
-      </c>
-      <c r="E35" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F35" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G35" s="12" t="inlineStr">
-        <is>
-          <t>AY GRİ Levha</t>
-        </is>
-      </c>
-      <c r="H35" s="17" t="inlineStr">
-        <is>
-          <t>WPC Levha Plaka</t>
-        </is>
-      </c>
-      <c r="I35" s="10" t="inlineStr">
-        <is>
-          <t>2.07 m</t>
-        </is>
-      </c>
-      <c r="J35" s="17" t="inlineStr">
-        <is>
-          <t>En: 94 cm (2 mm)</t>
-        </is>
-      </c>
-      <c r="K35" s="31" t="n">
-        <v>4.64</v>
-      </c>
-      <c r="L35" s="51" t="n">
-        <v>40</v>
-      </c>
-      <c r="M35" s="52" t="n">
-        <v>480</v>
-      </c>
-      <c r="N35" s="53" t="n">
-        <v>960</v>
-      </c>
-      <c r="O35" s="35" t="n">
-        <v>4454.4</v>
-      </c>
-      <c r="P35" s="36" t="inlineStr">
-        <is>
-          <t>480 Kapı/Gün</t>
-        </is>
-      </c>
-      <c r="Q35" s="37" t="inlineStr">
-        <is>
-          <t>Seri Üretim</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="38" t="inlineStr">
-        <is>
-          <t>↳ Hat 201 (Levha)</t>
-        </is>
-      </c>
-      <c r="B36" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C36" s="39" t="n">
-        <v>720</v>
-      </c>
-      <c r="D36" s="40" t="n">
-        <v>720</v>
-      </c>
-      <c r="E36" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F36" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G36" s="4" t="inlineStr">
-        <is>
-          <t>SONOMO Levha</t>
-        </is>
-      </c>
-      <c r="H36" s="9" t="inlineStr">
-        <is>
-          <t>WPC Levha Plaka</t>
-        </is>
-      </c>
-      <c r="I36" s="10" t="inlineStr">
-        <is>
-          <t>2.07 m</t>
-        </is>
-      </c>
-      <c r="J36" s="9" t="inlineStr">
-        <is>
-          <t>En: 94 cm (2 mm)</t>
-        </is>
-      </c>
-      <c r="K36" s="41" t="n">
-        <v>4.33</v>
-      </c>
-      <c r="L36" s="48" t="n">
-        <v>38.4</v>
-      </c>
-      <c r="M36" s="49" t="n">
-        <v>461</v>
-      </c>
-      <c r="N36" s="50" t="n">
-        <v>922</v>
-      </c>
-      <c r="O36" s="45" t="n">
-        <v>3992.3</v>
-      </c>
-      <c r="P36" s="46" t="inlineStr">
-        <is>
-          <t>461 Kapı/Gün</t>
-        </is>
-      </c>
-      <c r="Q36" s="38" t="inlineStr">
-        <is>
-          <t>Seri Üretim</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="20" customHeight="1">
-      <c r="A37" s="37" t="inlineStr">
-        <is>
-          <t>↳ Hat 201 (Levha)</t>
-        </is>
-      </c>
-      <c r="B37" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C37" s="28" t="n">
-        <v>720</v>
-      </c>
-      <c r="D37" s="29" t="n">
-        <v>720</v>
-      </c>
-      <c r="E37" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F37" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G37" s="12" t="inlineStr">
-        <is>
-          <t>COCO Levha</t>
-        </is>
-      </c>
-      <c r="H37" s="17" t="inlineStr">
-        <is>
-          <t>WPC Levha Plaka</t>
-        </is>
-      </c>
-      <c r="I37" s="10" t="inlineStr">
-        <is>
-          <t>2.07 m</t>
-        </is>
-      </c>
-      <c r="J37" s="17" t="inlineStr">
-        <is>
-          <t>En: 94 cm (2 mm)</t>
-        </is>
-      </c>
-      <c r="K37" s="31" t="n">
-        <v>4.79</v>
-      </c>
-      <c r="L37" s="51" t="n">
-        <v>41.4</v>
-      </c>
-      <c r="M37" s="52" t="n">
-        <v>497</v>
-      </c>
-      <c r="N37" s="53" t="n">
-        <v>994</v>
-      </c>
-      <c r="O37" s="35" t="n">
-        <v>4761.3</v>
-      </c>
-      <c r="P37" s="36" t="inlineStr">
-        <is>
-          <t>497 Kapı/Gün</t>
-        </is>
-      </c>
-      <c r="Q37" s="37" t="inlineStr">
-        <is>
-          <t>Seri Üretim</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="38" t="inlineStr">
-        <is>
-          <t>↳ Hat 201 (Levha)</t>
-        </is>
-      </c>
-      <c r="B38" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C38" s="39" t="n">
-        <v>720</v>
-      </c>
-      <c r="D38" s="40" t="n">
-        <v>720</v>
-      </c>
-      <c r="E38" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F38" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G38" s="4" t="inlineStr">
-        <is>
-          <t>ANTRASİT Levha</t>
-        </is>
-      </c>
-      <c r="H38" s="9" t="inlineStr">
-        <is>
-          <t>WPC Levha Plaka</t>
-        </is>
-      </c>
-      <c r="I38" s="10" t="inlineStr">
-        <is>
-          <t>2.07 m</t>
-        </is>
-      </c>
-      <c r="J38" s="9" t="inlineStr">
-        <is>
-          <t>En: 94 cm (2 mm)</t>
-        </is>
-      </c>
-      <c r="K38" s="41" t="n">
-        <v>4.77</v>
-      </c>
-      <c r="L38" s="48" t="n">
-        <v>40</v>
-      </c>
-      <c r="M38" s="49" t="n">
-        <v>480</v>
-      </c>
-      <c r="N38" s="50" t="n">
-        <v>960</v>
-      </c>
-      <c r="O38" s="45" t="n">
-        <v>4579.2</v>
-      </c>
-      <c r="P38" s="46" t="inlineStr">
-        <is>
-          <t>480 Kapı/Gün</t>
-        </is>
-      </c>
-      <c r="Q38" s="38" t="inlineStr">
-        <is>
-          <t>Seri Üretim</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="20" customHeight="1">
-      <c r="A39" s="37" t="inlineStr">
-        <is>
-          <t>↳ Hat 201 (Levha)</t>
-        </is>
-      </c>
-      <c r="B39" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C39" s="28" t="n">
-        <v>720</v>
-      </c>
-      <c r="D39" s="29" t="n">
-        <v>720</v>
-      </c>
-      <c r="E39" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F39" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G39" s="12" t="inlineStr">
-        <is>
-          <t>VIZON Levha</t>
-        </is>
-      </c>
-      <c r="H39" s="17" t="inlineStr">
-        <is>
-          <t>WPC Levha Plaka</t>
-        </is>
-      </c>
-      <c r="I39" s="10" t="inlineStr">
-        <is>
-          <t>2.07 m</t>
-        </is>
-      </c>
-      <c r="J39" s="17" t="inlineStr">
-        <is>
-          <t>En: 94 cm (2 mm)</t>
-        </is>
-      </c>
-      <c r="K39" s="31" t="n">
-        <v>4.77</v>
-      </c>
-      <c r="L39" s="51" t="n">
-        <v>34</v>
-      </c>
-      <c r="M39" s="52" t="n">
-        <v>408</v>
-      </c>
-      <c r="N39" s="53" t="n">
-        <v>816</v>
-      </c>
-      <c r="O39" s="35" t="n">
-        <v>3892.3</v>
-      </c>
-      <c r="P39" s="36" t="inlineStr">
-        <is>
-          <t>408 Kapı/Gün</t>
-        </is>
-      </c>
-      <c r="Q39" s="37" t="inlineStr">
-        <is>
-          <t>Seri Üretim</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="38" t="inlineStr">
-        <is>
-          <t>↳ Hat 201 (Levha)</t>
-        </is>
-      </c>
-      <c r="B40" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C40" s="39" t="n">
-        <v>720</v>
-      </c>
-      <c r="D40" s="40" t="n">
-        <v>720</v>
-      </c>
-      <c r="E40" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F40" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G40" s="4" t="inlineStr">
-        <is>
-          <t>KOYU CEVİZ Levha</t>
-        </is>
-      </c>
-      <c r="H40" s="9" t="inlineStr">
-        <is>
-          <t>WPC Levha Plaka</t>
-        </is>
-      </c>
-      <c r="I40" s="10" t="inlineStr">
-        <is>
-          <t>2.07 m</t>
-        </is>
-      </c>
-      <c r="J40" s="9" t="inlineStr">
-        <is>
-          <t>En: 94 cm (2 mm)</t>
-        </is>
-      </c>
-      <c r="K40" s="41" t="n">
-        <v>4.79</v>
-      </c>
-      <c r="L40" s="48" t="n">
-        <v>28.8</v>
-      </c>
-      <c r="M40" s="49" t="n">
-        <v>346</v>
-      </c>
-      <c r="N40" s="50" t="n">
-        <v>691</v>
-      </c>
-      <c r="O40" s="45" t="n">
-        <v>3309.9</v>
-      </c>
-      <c r="P40" s="46" t="inlineStr">
-        <is>
-          <t>346 Kapı/Gün</t>
-        </is>
-      </c>
-      <c r="Q40" s="38" t="inlineStr">
-        <is>
-          <t>Seri Üretim</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="20" customHeight="1">
-      <c r="A41" s="12" t="inlineStr">
-        <is>
-          <t>KALİTE KONTROL</t>
-        </is>
-      </c>
-      <c r="B41" s="13" t="inlineStr">
-        <is>
-          <t>08:30 / 20:30 (2V)</t>
-        </is>
-      </c>
-      <c r="C41" s="28" t="n">
-        <v>720</v>
-      </c>
-      <c r="D41" s="29" t="n">
-        <v>720</v>
-      </c>
-      <c r="E41" s="30" t="n">
-        <v>3</v>
-      </c>
-      <c r="F41" s="30" t="n">
-        <v>3</v>
-      </c>
-      <c r="G41" s="12" t="inlineStr">
-        <is>
-          <t>TÜM PROFİL &amp; LEVHALAR</t>
-        </is>
-      </c>
-      <c r="H41" s="17" t="inlineStr">
-        <is>
-          <t>Kalite Güvence</t>
-        </is>
-      </c>
-      <c r="I41" s="10" t="inlineStr">
-        <is>
-          <t>Tüm Boylar</t>
-        </is>
-      </c>
-      <c r="J41" s="17" t="inlineStr">
-        <is>
-          <t>Tüm Kesitler</t>
-        </is>
-      </c>
-      <c r="K41" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L41" s="54" t="n">
-        <v>175</v>
-      </c>
-      <c r="M41" s="55" t="n">
-        <v>2100</v>
-      </c>
-      <c r="N41" s="56" t="n">
-        <v>4200</v>
-      </c>
-      <c r="O41" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P41" s="14" t="inlineStr">
-        <is>
-          <t>4.200 Adet/Gün</t>
-        </is>
-      </c>
-      <c r="Q41" s="37" t="inlineStr">
-        <is>
           <t>Son Kontrol</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="24" customHeight="1">
-      <c r="A42" s="57" t="inlineStr">
+    <row r="32" ht="24" customHeight="1">
+      <c r="A32" s="54" t="inlineStr">
         <is>
           <t>GENEL TOPLAM (FİLTREYE DUYARLI)</t>
         </is>
       </c>
-      <c r="B42" s="22" t="n"/>
-      <c r="C42" s="22" t="n"/>
-      <c r="D42" s="22" t="n"/>
-      <c r="E42" s="22" t="n"/>
-      <c r="F42" s="22" t="n"/>
-      <c r="G42" s="22" t="n"/>
-      <c r="H42" s="22" t="n"/>
-      <c r="I42" s="22" t="n"/>
-      <c r="J42" s="22" t="n"/>
-      <c r="K42" s="22" t="n"/>
-      <c r="L42" s="22" t="n"/>
-      <c r="M42" s="58">
-        <f>SUBTOTAL(109, M5:M41)</f>
+      <c r="B32" s="22" t="n"/>
+      <c r="C32" s="22" t="n"/>
+      <c r="D32" s="22" t="n"/>
+      <c r="E32" s="22" t="n"/>
+      <c r="F32" s="22" t="n"/>
+      <c r="G32" s="22" t="n"/>
+      <c r="H32" s="22" t="n"/>
+      <c r="I32" s="22" t="n"/>
+      <c r="J32" s="22" t="n"/>
+      <c r="K32" s="22" t="n"/>
+      <c r="L32" s="22" t="n"/>
+      <c r="M32" s="55">
+        <f>SUBTOTAL(109, M5:M31)</f>
         <v/>
       </c>
-      <c r="N42" s="58">
-        <f>SUBTOTAL(109, N5:N41)</f>
+      <c r="N32" s="55">
+        <f>SUBTOTAL(109, N5:N31)</f>
         <v/>
       </c>
-      <c r="O42" s="22" t="n"/>
-      <c r="P42" s="22" t="n"/>
-      <c r="Q42" s="22" t="n"/>
+      <c r="O32" s="22" t="n"/>
+      <c r="P32" s="22" t="n"/>
+      <c r="Q32" s="22" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:Q41"/>
+  <autoFilter ref="A4:Q31"/>
   <mergeCells count="5">
     <mergeCell ref="G3:K3"/>
     <mergeCell ref="A2:Q2"/>

</xml_diff>